<commit_message>
Phase 4 + research: verified Rule Book, real-remark decoder eval, Temporal cycle, voice, i18n, benchmarks
- Rule Book checked against official sources (EPF Scheme 2026, Rs 25,000 wage ceiling, 12-month
  final-settlement wait, partial-withdrawal reform); every rule carries its source; 10 new rules
- 148 real public EPFO remarks (test-only); decoder taxonomy 15 -> 20 categories; retrained on
  Tinker (v3): 72% vs 58% base vs 53% Gemma few-shot on real remarks
- Temporal MonthlyCycle + ClaimFollowUp workflows, salary sheet validation, Cycle page;
  kill-resume 20/20 after fixing a late-sheet bug the test found
- Helpline: rejected-claim fixed reply, foreign-script retry; ElevenLabs custom-LLM endpoint + widget
- Hindi/Marathi UI toggle; Sentry spans (metadata only); benchmarks for pre-check, search, helpline

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/PF_Desk_Papa_Template.xlsx
+++ b/docs/PF_Desk_Papa_Template.xlsx
@@ -11047,7 +11047,7 @@
       <formula2>1000</formula2>
     </dataValidation>
     <dataValidation sqref="E4:E503" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="List se chunein" error="Neeche ke arrow se list me se chunein." type="list">
-      <formula1>='Lists'!$C$2:$C$16</formula1>
+      <formula1>='Lists'!$C$2:$C$21</formula1>
     </dataValidation>
     <dataValidation sqref="F4:F503" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="List se chunein" error="Neeche ke arrow se list me se chunein." type="list">
       <formula1>='Lists'!$D$2:$D$4</formula1>
@@ -13657,7 +13657,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B4:B503" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="List se chunein" error="Neeche ke arrow se list me se chunein." type="list">
-      <formula1>='Lists'!$M$2:$M$16</formula1>
+      <formula1>='Lists'!$M$2:$M$21</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13671,7 +13671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14102,10 +14102,70 @@
     <row r="16">
       <c r="C16" s="16" t="inlineStr">
         <is>
+          <t>Pension (EPS) ki problem</t>
+        </is>
+      </c>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>Pension (EPS) ki problem</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Contribution nahi aaya / ECR reconcile nahi</t>
+        </is>
+      </c>
+      <c r="M17" s="16" t="inlineStr">
+        <is>
+          <t>Contribution nahi aaya / ECR reconcile nahi</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>Purani naukri ka transfer pending</t>
+        </is>
+      </c>
+      <c r="M18" s="16" t="inlineStr">
+        <is>
+          <t>Purani naukri ka transfer pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>PAN / Form 15G / TDS</t>
+        </is>
+      </c>
+      <c r="M19" s="16" t="inlineStr">
+        <is>
+          <t>PAN / Form 15G / TDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Employer ka confirmation / genuineness letter</t>
+        </is>
+      </c>
+      <c r="M20" s="16" t="inlineStr">
+        <is>
+          <t>Employer ka confirmation / genuineness letter</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" s="16" t="inlineStr">
+        <is>
           <t>Kuch aur (Note me likhein)</t>
         </is>
       </c>
-      <c r="M16" s="16" t="inlineStr">
+      <c r="M21" s="16" t="inlineStr">
         <is>
           <t>Kuch aur (Note me likhein)</t>
         </is>

</xml_diff>